<commit_message>
Cash sales: import MS into new "Cash MS" type, numbered by date
MS cash sales now go to the new Tally voucher type "Cash MS" and each
voucher is numbered by its date (Cash/MS/1Oct2026), so no starting number
is needed. The hand-entered "MS Cash" type is never touched. Two MS rows
on the same day are refused (they would share a number) with a message to
combine them. HSD and XG still continue from the starting numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XEsSP5YnaquLgj2FgxycqU
</commit_message>
<xml_diff>
--- a/fleet_tally/samples/cash_sales_template.xlsx
+++ b/fleet_tally/samples/cash_sales_template.xlsx
@@ -454,14 +454,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cash sales — Motor Spirit (petrol)  →  Tally voucher type “MS Cash” (CASH/MS/…)</t>
+          <t>Cash sales — Motor Spirit (petrol)  →  Tally voucher type “Cash MS” (numbered by date: Cash/MS/1Oct2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per day: the litres sold for cash and that day's price per litre. Amount = Quantity × Price (rounded to paise). Leave a day out if nothing was sold.</t>
+          <t>One row per day (the voucher number is the date): the litres sold for cash and that day's price per litre. Amount = Quantity × Price (rounded to paise). Leave a day out if nothing was sold.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cash sales: number HSD CASH and XG CASH vouchers by date too
HSD and XG cash vouchers are now numbered like Cash MS: Cash/HSD/1Oct2026,
Cash/XG/1Oct2026. They still import into the existing HSD CASH / XG CASH
voucher types. With every product numbered by date, the starting-number
boxes and the saved cash_start are gone; two rows of the same product on
one day are refused with a message to combine them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XEsSP5YnaquLgj2FgxycqU
</commit_message>
<xml_diff>
--- a/fleet_tally/samples/cash_sales_template.xlsx
+++ b/fleet_tally/samples/cash_sales_template.xlsx
@@ -684,14 +684,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cash sales — High Speed Diesel  →  Tally voucher type “HSD CASH” (CASH/HSD/…)</t>
+          <t>Cash sales — High Speed Diesel  →  Tally voucher type “HSD CASH” (numbered by date: Cash/HSD/1Oct2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per day: the litres sold for cash and that day's price per litre. Amount = Quantity × Price (rounded to paise). Leave a day out if nothing was sold.</t>
+          <t>One row per day (the voucher number is the date): the litres sold for cash and that day's price per litre. Amount = Quantity × Price (rounded to paise). Leave a day out if nothing was sold.</t>
         </is>
       </c>
     </row>
@@ -914,14 +914,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cash sales — XtraGreen Diesel  →  Tally voucher type “XG CASH” (CASH/XG/…)</t>
+          <t>Cash sales — XtraGreen Diesel  →  Tally voucher type “XG CASH” (numbered by date: Cash/XG/1Oct2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per day: the litres sold for cash and that day's price per litre. Amount = Quantity × Price (rounded to paise). Leave a day out if nothing was sold.</t>
+          <t>One row per day (the voucher number is the date): the litres sold for cash and that day's price per litre. Amount = Quantity × Price (rounded to paise). Leave a day out if nothing was sold.</t>
         </is>
       </c>
     </row>

</xml_diff>